<commit_message>
working on effectiveness report
</commit_message>
<xml_diff>
--- a/application/plugins/Reports_summary_sell_stock/Reports_summary_sell_stock.xlsx
+++ b/application/plugins/Reports_summary_sell_stock/Reports_summary_sell_stock.xlsx
@@ -9,12 +9,12 @@
   <sheets>
     <sheet name="Отчет" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
   <si>
     <t>{$v-&gt;rows[]-&gt;group_by}</t>
   </si>
@@ -101,12 +101,21 @@
   </si>
   <si>
     <t>сумма</t>
+  </si>
+  <si>
+    <t>{$v-&gt;summary_rows[]-&gt;sellout_days}</t>
+  </si>
+  <si>
+    <t>Запас дней</t>
+  </si>
+  <si>
+    <t>{$v-&gt;total_stock_sellout}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -141,7 +150,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -160,8 +169,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF93CDDD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="18">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -312,7 +333,57 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -326,28 +397,6 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -361,7 +410,9 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -373,7 +424,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -400,9 +451,6 @@
     <xf numFmtId="2" fontId="2" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -415,7 +463,7 @@
     <xf numFmtId="1" fontId="2" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -424,70 +472,87 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
-    <cellStyle name="Процентный" xfId="1" builtinId="5"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF2F2F2"/>
+      <color rgb="FF93CDDD"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -500,9 +565,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -540,7 +605,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -612,7 +677,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -795,64 +860,68 @@
   <sheetData>
     <row r="1" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="28"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="23"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="21"/>
-      <c r="D3" s="29" t="s">
+      <c r="C3" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="29" t="s">
+      <c r="E3" s="33"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="30"/>
-      <c r="I3" s="32"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="35"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B4" s="22"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="12" t="s">
+      <c r="B4" s="36"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="H4" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="40" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="36"/>
+      <c r="C5" s="42" t="s">
+        <v>31</v>
+      </c>
       <c r="D5" s="8">
         <v>1</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="14" t="s">
         <v>10</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -861,7 +930,7 @@
       <c r="G5" s="10">
         <v>1</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="15" t="s">
         <v>11</v>
       </c>
       <c r="I5" s="11" t="s">
@@ -869,10 +938,12 @@
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="25"/>
+      <c r="C6" s="41" t="s">
+        <v>29</v>
+      </c>
       <c r="D6" s="5" t="s">
         <v>19</v>
       </c>
@@ -904,66 +975,66 @@
     </row>
     <row r="9" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="10" spans="2:9" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="28"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="23"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="D11" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="34"/>
-      <c r="F11" s="37" t="s">
+      <c r="E11" s="25"/>
+      <c r="F11" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="G11" s="37"/>
-      <c r="H11" s="37" t="s">
+      <c r="G11" s="28"/>
+      <c r="H11" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="I11" s="38"/>
+      <c r="I11" s="29"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B12" s="22"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="13" t="s">
+      <c r="B12" s="27"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="G12" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I12" s="14" t="s">
+      <c r="I12" s="13" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="33" t="s">
+      <c r="D13" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="33"/>
+      <c r="E13" s="24"/>
       <c r="F13" s="7" t="s">
         <v>16</v>
       </c>
@@ -973,7 +1044,7 @@
       <c r="H13" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="I13" s="19" t="s">
+      <c r="I13" s="18" t="s">
         <v>15</v>
       </c>
     </row>
@@ -988,20 +1059,19 @@
       <c r="I14" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="12">
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="G3:I3"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="D11:E12"/>
     <mergeCell ref="C11:C12"/>
     <mergeCell ref="B11:B12"/>
-    <mergeCell ref="B5:C5"/>
     <mergeCell ref="B10:I10"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="F11:G11"/>
-    <mergeCell ref="B3:C4"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>